<commit_message>
Login and SignUp TestCase Done
</commit_message>
<xml_diff>
--- a/test-data/Test-Data.xlsx
+++ b/test-data/Test-Data.xlsx
@@ -1,13 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation Testing Pipeline\test-data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{133CEEAD-2BC3-49CF-B9B1-A928C61F10BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="SignUp" sheetId="2" r:id="rId1"/>
+    <sheet name="Login" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,12 +25,72 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>expected</t>
+  </si>
+  <si>
+    <t>TestName</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>yashsabhani1234@gmail.com</t>
+  </si>
+  <si>
+    <t>Testing12</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>RAJACHOMUCHAND@gmail.com</t>
+  </si>
+  <si>
+    <t>Sign Up</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>RAJA_Moli_3249</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -37,7 +104,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,14 +112,54 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,10 +437,95 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30EC72F2-9FBF-47E6-A6CA-228AD99F6210}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.90625" customWidth="1"/>
+    <col min="2" max="2" width="12.1796875" customWidth="1"/>
+    <col min="3" max="3" width="28.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.90625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{8CA5A7B5-4290-4A1E-B3E9-6254E3AC61D6}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.36328125" customWidth="1"/>
+    <col min="2" max="2" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" tooltip="mailto:yashsabhani1234@gmail.com" display="mailto:yashsabhani1234@gmail.com" xr:uid="{3987526B-03BD-4EE3-8110-1ABAE2B3D406}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>